<commit_message>
add exclude + use pull()
</commit_message>
<xml_diff>
--- a/paper/data/exclude.xlsx
+++ b/paper/data/exclude.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tilburgu-my.sharepoint.com/personal/s_m_ostergaard_tilburguniversity_edu/Documents/PhD/self-paced_eeg/natural-stories-dutch/paper/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="11_F25DC773A252ABDACC10482BD19F64965BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{763E5217-884A-4FB8-A970-DACC0721FB8F}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="11_F25DC773A252ABDACC10482BD19F64965BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE24A8E1-10BC-4450-9320-B641DA72B575}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
   <si>
     <t>ch</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t>AFz</t>
+  </si>
+  <si>
+    <t>TP7</t>
   </si>
 </sst>
 </file>
@@ -391,7 +394,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.26953125" customWidth="1"/>
@@ -416,46 +419,40 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>17</v>
-      </c>
-      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>25</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -463,7 +460,7 @@
         <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -474,7 +471,7 @@
         <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
@@ -485,7 +482,7 @@
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
@@ -496,7 +493,7 @@
         <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
@@ -504,10 +501,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -515,12 +512,34 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12">
         <v>26</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
         <v>7</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D13" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>